<commit_message>
- add it staff download
</commit_message>
<xml_diff>
--- a/app/static/uploads/list.xlsx
+++ b/app/static/uploads/list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PERSONAL_DEVELOPMENT\PROJECTS\INVIGILATOR\app\static\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE8E2AA-B734-4D9B-8D61-77C08B06B0FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A5E1BE-BADA-4149-BACD-DB2058AA5137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29280" yWindow="1050" windowWidth="27555" windowHeight="15480" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="269">
   <si>
     <t>title</t>
   </si>
@@ -1217,6 +1217,9 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>105</v>
+      </c>
       <c r="B4" t="s">
         <v>15</v>
       </c>
@@ -1234,6 +1237,9 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -1251,6 +1257,9 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
       <c r="B6" t="s">
         <v>266</v>
       </c>
@@ -1268,6 +1277,9 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
       <c r="B7" t="s">
         <v>22</v>
       </c>
@@ -1305,6 +1317,9 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
       <c r="B9" t="s">
         <v>30</v>
       </c>
@@ -1336,6 +1351,9 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
       <c r="B11" t="s">
         <v>36</v>
       </c>
@@ -1370,6 +1388,9 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>105</v>
+      </c>
       <c r="B13" t="s">
         <v>41</v>
       </c>
@@ -1387,6 +1408,9 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>105</v>
+      </c>
       <c r="B14" t="s">
         <v>43</v>
       </c>
@@ -1404,6 +1428,9 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>105</v>
+      </c>
       <c r="B15" t="s">
         <v>47</v>
       </c>
@@ -1472,6 +1499,9 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
       <c r="B19" t="s">
         <v>56</v>
       </c>
@@ -1506,6 +1536,9 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
       <c r="B21" t="s">
         <v>60</v>
       </c>
@@ -1523,6 +1556,9 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>24</v>
+      </c>
       <c r="B22" t="s">
         <v>62</v>
       </c>
@@ -1560,6 +1596,9 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
       <c r="B24" t="s">
         <v>67</v>
       </c>
@@ -1628,6 +1667,9 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>24</v>
+      </c>
       <c r="B28" t="s">
         <v>77</v>
       </c>
@@ -1662,6 +1704,9 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>105</v>
+      </c>
       <c r="B30" t="s">
         <v>84</v>
       </c>
@@ -1696,6 +1741,9 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>24</v>
+      </c>
       <c r="B32" t="s">
         <v>88</v>
       </c>
@@ -1744,6 +1792,9 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>105</v>
+      </c>
       <c r="B35" t="s">
         <v>94</v>
       </c>
@@ -1761,6 +1812,9 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>24</v>
+      </c>
       <c r="B36" t="s">
         <v>96</v>
       </c>
@@ -1812,6 +1866,9 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
       <c r="B39" t="s">
         <v>100</v>
       </c>
@@ -1897,6 +1954,9 @@
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>24</v>
+      </c>
       <c r="B44" t="s">
         <v>113</v>
       </c>
@@ -1948,6 +2008,9 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>24</v>
+      </c>
       <c r="B47" t="s">
         <v>121</v>
       </c>
@@ -1979,6 +2042,9 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>24</v>
+      </c>
       <c r="B49" t="s">
         <v>123</v>
       </c>
@@ -2013,6 +2079,9 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>24</v>
+      </c>
       <c r="B51" t="s">
         <v>129</v>
       </c>
@@ -2047,6 +2116,9 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>24</v>
+      </c>
       <c r="B53" t="s">
         <v>133</v>
       </c>
@@ -2081,6 +2153,9 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>24</v>
+      </c>
       <c r="B55" t="s">
         <v>137</v>
       </c>
@@ -2129,6 +2204,9 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>108</v>
+      </c>
       <c r="B58" t="s">
         <v>143</v>
       </c>
@@ -2180,6 +2258,9 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>24</v>
+      </c>
       <c r="B61" t="s">
         <v>150</v>
       </c>
@@ -2197,6 +2278,9 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>105</v>
+      </c>
       <c r="B62" t="s">
         <v>152</v>
       </c>
@@ -2214,6 +2298,9 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>24</v>
+      </c>
       <c r="B63" t="s">
         <v>154</v>
       </c>
@@ -2245,6 +2332,9 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>105</v>
+      </c>
       <c r="B65" t="s">
         <v>159</v>
       </c>
@@ -2347,6 +2437,9 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>24</v>
+      </c>
       <c r="B71" t="s">
         <v>165</v>
       </c>
@@ -2364,6 +2457,9 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>6</v>
+      </c>
       <c r="B72" t="s">
         <v>170</v>
       </c>
@@ -2395,6 +2491,9 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>6</v>
+      </c>
       <c r="B74" t="s">
         <v>174</v>
       </c>
@@ -2409,6 +2508,9 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>24</v>
+      </c>
       <c r="B75" t="s">
         <v>177</v>
       </c>
@@ -2460,6 +2562,9 @@
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>24</v>
+      </c>
       <c r="B78" t="s">
         <v>182</v>
       </c>
@@ -2477,6 +2582,9 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>24</v>
+      </c>
       <c r="B79" t="s">
         <v>184</v>
       </c>
@@ -2511,6 +2619,9 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>24</v>
+      </c>
       <c r="B81" t="s">
         <v>188</v>
       </c>
@@ -2562,6 +2673,9 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>108</v>
+      </c>
       <c r="B84" t="s">
         <v>191</v>
       </c>
@@ -2593,6 +2707,9 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>105</v>
+      </c>
       <c r="B86" t="s">
         <v>195</v>
       </c>
@@ -2610,6 +2727,9 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>24</v>
+      </c>
       <c r="B87" t="s">
         <v>121</v>
       </c>
@@ -2627,6 +2747,9 @@
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>24</v>
+      </c>
       <c r="B88" t="s">
         <v>121</v>
       </c>
@@ -2712,6 +2835,9 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>24</v>
+      </c>
       <c r="B93" t="s">
         <v>206</v>
       </c>
@@ -2777,6 +2903,9 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>24</v>
+      </c>
       <c r="B97" t="s">
         <v>212</v>
       </c>
@@ -2845,6 +2974,9 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>24</v>
+      </c>
       <c r="B101" t="s">
         <v>214</v>
       </c>
@@ -2896,6 +3028,9 @@
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>24</v>
+      </c>
       <c r="B104" t="s">
         <v>214</v>
       </c>
@@ -3015,6 +3150,9 @@
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>105</v>
+      </c>
       <c r="B111" t="s">
         <v>236</v>
       </c>
@@ -3029,6 +3167,9 @@
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>24</v>
+      </c>
       <c r="B112" t="s">
         <v>238</v>
       </c>
@@ -3043,6 +3184,9 @@
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>24</v>
+      </c>
       <c r="B113" t="s">
         <v>240</v>
       </c>
@@ -3142,6 +3286,9 @@
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>24</v>
+      </c>
       <c r="B119" t="s">
         <v>251</v>
       </c>
@@ -3190,6 +3337,9 @@
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>24</v>
+      </c>
       <c r="B122" t="s">
         <v>256</v>
       </c>
@@ -3204,6 +3354,9 @@
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>24</v>
+      </c>
       <c r="B123" t="s">
         <v>257</v>
       </c>
@@ -3272,6 +3425,9 @@
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>24</v>
+      </c>
       <c r="B127" t="s">
         <v>264</v>
       </c>

</xml_diff>